<commit_message>
Adding explanations to each section
</commit_message>
<xml_diff>
--- a/exports/prerelease_participants.xlsx
+++ b/exports/prerelease_participants.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,144 +443,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Test User 1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>sg123456789</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>11112222</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Test User 2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>sg223456789</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>00009999</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Test User 3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>sg32345678</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>33334444</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>729</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Test User 4</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>sg42345678</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>55556666</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Test User 5</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>sg52345678</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>77778888</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Test User 6</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>sg98765432</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>12345678</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>446</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>